<commit_message>
Update security audit register: add Status column with remediation state
Add a color-coded Status (fix ref) column to the Audit To-Dos sheet mapping each
finding to its commit or state, and refresh the subtitle with the remediation
snapshot. 16 of 21 fixed; SEC-05 parked (owner), SEC-15 plan-first, SEC-19/20
open, SEC-21 partial.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SzJ77UAHhR8QZAy3qQhqq3
</commit_message>
<xml_diff>
--- a/AureonCare_Security_Audit_ToDos.xlsx
+++ b/AureonCare_Security_Audit_ToDos.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,8 +74,24 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="009C5700"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +128,21 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -139,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -187,6 +218,15 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -553,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -566,6 +606,7 @@
     <col width="44" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -578,7 +619,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Read-only audit performed 2026-08-01 on branch claude/security-audit-impact-vEc4g. No code changed. Severity = exploitability x data sensitivity (PHI). 'Impacted Modules' lists the coordinated/linked changes each fix pulls in.</t>
+          <t>Audit performed 2026-08-01 on branch claude/security-audit-impact-vEc4g. Remediation status updated 2026-08-14 (Status column). 16 of 21 fixed; SEC-05 parked (owner), SEC-15 plan-first, SEC-19/20 open, SEC-21 partial. Severity = exploitability x data sensitivity (PHI).</t>
         </is>
       </c>
     </row>
@@ -633,6 +674,11 @@
           <t>Priority</t>
         </is>
       </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Status (fix ref)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="78" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -685,6 +731,11 @@
           <t>P0</t>
         </is>
       </c>
+      <c r="K5" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — 5414409</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="78" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -737,6 +788,11 @@
           <t>P0</t>
         </is>
       </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — 5414409</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="78" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -789,6 +845,11 @@
           <t>P0</t>
         </is>
       </c>
+      <c r="K7" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — 5414409</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -841,6 +902,11 @@
           <t>P0</t>
         </is>
       </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — 5414409 + 3c9cfa0</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="78" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -893,6 +959,11 @@
           <t>P1</t>
         </is>
       </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>⏸ Parked — deferred by owner — XL multi-tenant scoping</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="78" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -945,6 +1016,11 @@
           <t>P1</t>
         </is>
       </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — 2a78980</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="78" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -997,6 +1073,11 @@
           <t>P1</t>
         </is>
       </c>
+      <c r="K11" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — 2a78980</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="78" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -1049,6 +1130,11 @@
           <t>P1</t>
         </is>
       </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — 2a78980</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="78" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -1101,6 +1187,11 @@
           <t>P2</t>
         </is>
       </c>
+      <c r="K13" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — e4038cb</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="78" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -1153,6 +1244,11 @@
           <t>P2</t>
         </is>
       </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — e4038cb</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="78" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1205,6 +1301,11 @@
           <t>P2</t>
         </is>
       </c>
+      <c r="K15" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — e4038cb</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="78" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -1257,6 +1358,11 @@
           <t>P2</t>
         </is>
       </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — ca06b7f — breach/HIBP check deferred</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="78" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -1309,6 +1415,11 @@
           <t>P2</t>
         </is>
       </c>
+      <c r="K17" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — ca06b7f</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="78" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -1361,6 +1472,11 @@
           <t>P2</t>
         </is>
       </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — ca06b7f</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="78" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -1413,6 +1529,11 @@
           <t>P2</t>
         </is>
       </c>
+      <c r="K19" s="19" t="inlineStr">
+        <is>
+          <t>▷ Plan-first — L — cookie/CSRF migration; plan pending sign-off</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="78" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
@@ -1465,6 +1586,11 @@
           <t>P2</t>
         </is>
       </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — e4038cb</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="78" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -1517,6 +1643,11 @@
           <t>P3</t>
         </is>
       </c>
+      <c r="K21" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — ca06b7f</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="78" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
@@ -1569,6 +1700,11 @@
           <t>P3</t>
         </is>
       </c>
+      <c r="K22" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — e4038cb</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="78" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -1621,6 +1757,11 @@
           <t>P3</t>
         </is>
       </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>○ Open — not yet batched</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="78" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
@@ -1673,6 +1814,11 @@
           <t>P3</t>
         </is>
       </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>○ Open — not yet batched</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="78" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -1725,11 +1871,17 @@
           <t>P3</t>
         </is>
       </c>
+      <c r="K25" s="19" t="inlineStr">
+        <is>
+          <t>◑ Partial — global+auth+portal limiters shipped (Fix #10/#24); infra note open</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:J25"/>
-  <mergeCells count="1">
-    <mergeCell ref="A2:J2"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Register: SEC-05 plan-ready with Model D recommendation; mark SEC-19 fixed
SEC-05 status -> Plan-ready, recommending Model D (schema-per-tenant + control
plane) per SEC-05_MULTI_TENANCY_PLAN.md, pending model sign-off (Q1-Q4); pointer
added to its Recommended To-Do. SEC-19 status -> Fixed (edd66af + 03c7c8a).
Subtitle refreshed: 17 of 21 fixed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SzJ77UAHhR8QZAy3qQhqq3
</commit_message>
<xml_diff>
--- a/AureonCare_Security_Audit_ToDos.xlsx
+++ b/AureonCare_Security_Audit_ToDos.xlsx
@@ -619,7 +619,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Audit performed 2026-08-01 on branch claude/security-audit-impact-vEc4g. Remediation status updated 2026-08-14 (Status column). 16 of 21 fixed; SEC-05 parked (owner), SEC-15 plan-first, SEC-19/20 open, SEC-21 partial. Severity = exploitability x data sensitivity (PHI).</t>
+          <t>Audit performed 2026-08-01 on branch claude/security-audit-impact-vEc4g. Status updated 2026-08-18. 17 of 21 fixed (SEC-01..04,06..14,16..19); SEC-05 plan-ready (Model D recommended, see SEC-05_MULTI_TENANCY_PLAN.md); SEC-15 plan-first; SEC-20 held; SEC-21 partial. Severity = exploitability x data sensitivity (PHI).</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Introduce clinic/org scoping (column + WHERE clause) on all PHI tables &amp; queries, derived from req.user. Confirm whether product is multi-tenant.</t>
+          <t>Introduce clinic/org scoping (column + WHERE clause) on all PHI tables &amp; queries, derived from req.user. Confirm whether product is multi-tenant. | PLAN: SEC-05_MULTI_TENANCY_PLAN.md — recommend Model D (schema-per-tenant + control plane) for isolation with release-safe config/data; alternatives A (silo) / C (pool+RLS).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="K9" s="19" t="inlineStr">
         <is>
-          <t>⏸ Parked — deferred by owner — XL multi-tenant scoping</t>
+          <t>▷ Plan-ready — Model D (schema-per-tenant) recommended; see SEC-05_MULTI_TENANCY_PLAN.md; awaiting model sign-off (Q1–Q4)</t>
         </is>
       </c>
     </row>
@@ -1757,9 +1757,9 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="K23" s="20" t="inlineStr">
-        <is>
-          <t>○ Open — not yet batched</t>
+      <c r="K23" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed — edd66af (canonical-id match) + 03c7c8a (verified-email re-link keeps existing OAuth users working)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: SEC-05 delivered via Model D; refresh status to 18 of 21
SEC-05 marked implemented — schema-per-tenant multi-tenancy is built and tested:
control plane, 78-table cutover, full route sweep, identity scoping by practice_id,
hardened portal routing, least-privilege DB role, cross-tenant test suite and CI guard.
Deployment of migrations 063-074 plus AC_DB_U / AC_IDX_K configuration remains.

Also restates the three genuinely open items (SEC-15 plan-first, SEC-20 awaiting a
scope decision, SEC-21 partial) and re-surfaces the SSRF deep-review of calendar-sync /
integrationOAuth / backupProviders, which the original audit flagged as unfinished and
which has never been revisited.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SzJ77UAHhR8QZAy3qQhqq3
</commit_message>
<xml_diff>
--- a/AureonCare_Security_Audit_ToDos.xlsx
+++ b/AureonCare_Security_Audit_ToDos.xlsx
@@ -619,7 +619,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Audit performed 2026-08-01 on branch claude/security-audit-impact-vEc4g. Status updated 2026-08-18. 17 of 21 fixed (SEC-01..04,06..14,16..19); SEC-05 plan-ready (Model D recommended, see SEC-05_MULTI_TENANCY_PLAN.md); SEC-15 plan-first; SEC-20 held; SEC-21 partial. Severity = exploitability x data sensitivity (PHI).</t>
+          <t>Audit performed 2026-08-01 on branch claude/security-audit-impact-vEc4g. Status updated 2026-09-02. 18 of 21 fixed (SEC-01..14, 16..19 + SEC-05 delivered via Model D multi-tenancy). Open: SEC-15 (plan-first), SEC-20 (awaiting decision), SEC-21 (partial). Also outstanding from the original audit: SSRF deep-review of calendar-sync / integrationOAuth / backupProviders. Severity = exploitability x data sensitivity (PHI).</t>
         </is>
       </c>
     </row>
@@ -959,9 +959,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K9" s="19" t="inlineStr">
-        <is>
-          <t>▷ Plan-ready — Model D (schema-per-tenant) recommended; see SEC-05_MULTI_TENANCY_PLAN.md; awaiting model sign-off (Q1–Q4)</t>
+      <c r="K9" s="18" t="inlineStr">
+        <is>
+          <t>✔ Fixed (implemented) — Model D schema-per-tenant delivered: control plane, 78-table cutover, full route sweep, identity scoping by practice_id, hardened portal routing, least-privilege DB role, cross-tenant tests + CI guard. Remaining: deploy migrations 063-074 and set AC_DB_U/AC_IDX_K.</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="K19" s="19" t="inlineStr">
         <is>
-          <t>▷ Plan-first — L — cookie/CSRF migration; plan pending sign-off</t>
+          <t>▷ Plan-first — sessionStorage -&gt; HttpOnly cookies + CSRF. Not started (L).</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="K24" s="20" t="inlineStr">
         <is>
-          <t>○ Open — not yet batched</t>
+          <t>○ Open — implicit OAuth -&gt; authorization-code flow. Awaiting scope decision (Google-now vs plan-only vs park).</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="K25" s="19" t="inlineStr">
         <is>
-          <t>◑ Partial — global+auth+portal limiters shipped (Fix #10/#24); infra note open</t>
+          <t>◑ Partial — global/auth/portal rate limiters shipped (Fix #10/#24); infra-level note still open.</t>
         </is>
       </c>
     </row>

</xml_diff>